<commit_message>
Fase 5: análise fiscal multi-renda + aba Panorama na planilha
- Documento 05: classifica as 4 fontes de renda (Airbnb, outro aluguel PF, MEI,
  bolsa de mestrado), corrige a conclusão de IR, e sinaliza regularização do
  aluguel recebido há 4 anos via denúncia espontânea
- Planilha: nova aba "Panorama de Rendas" consolidando todas as fontes
  (tributável x isento) frente à isenção de R$5.000; coluna de outro aluguel

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011VkMFb5sFAokiKv7icQfpZ
</commit_message>
<xml_diff>
--- a/docs/fase-5-financeiro/controle-fiscal-airbnb.xlsx
+++ b/docs/fase-5-financeiro/controle-fiscal-airbnb.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Tabela IR" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Lançamentos Mensais" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Resumo Anual" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Panorama de Rendas" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -128,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -154,6 +155,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -960,8 +964,8 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Outros rendim.
-tributáveis R$</t>
+          <t>Outro aluguel
+(PF) tributável R$</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
@@ -1897,4 +1901,643 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>PANORAMA DE RENDAS (mensal) — todas as fontes e a isenção de R$ 5.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Tributável (entra na conta do IR) x Isento (não entra). Amarelo = você preenche; cinza = calculado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Presunção de lucro do MEI (serviços 32% / comércio 8% / transporte 16%):</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Mês</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Airbnb base
+tributável R$</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Outro aluguel
+tributável R$</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>MEI faturamento
+R$</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>MEI isento
+(presunção) R$</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>MEI parcela
+tributável R$</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Bolsa mestrado
+(isenta) R$</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL TRIBUTÁVEL
+mês R$</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL ISENTO
+mês R$</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Situação vs isenção
+R$ 5.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Janeiro</t>
+        </is>
+      </c>
+      <c r="B6" s="12">
+        <f>'Lançamentos Mensais'!L4</f>
+        <v/>
+      </c>
+      <c r="C6" s="12">
+        <f>'Lançamentos Mensais'!I4</f>
+        <v/>
+      </c>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="12">
+        <f>D6*$D$3</f>
+        <v/>
+      </c>
+      <c r="F6" s="12">
+        <f>MAX(0,D6-E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="13">
+        <f>B6+C6+F6</f>
+        <v/>
+      </c>
+      <c r="I6" s="13">
+        <f>E6+G6</f>
+        <v/>
+      </c>
+      <c r="J6" s="21">
+        <f>IF(H6=0,"-",IF(H6&lt;=5000,"Isento",IF(H6&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Fevereiro</t>
+        </is>
+      </c>
+      <c r="B7" s="12">
+        <f>'Lançamentos Mensais'!L5</f>
+        <v/>
+      </c>
+      <c r="C7" s="12">
+        <f>'Lançamentos Mensais'!I5</f>
+        <v/>
+      </c>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="12">
+        <f>D7*$D$3</f>
+        <v/>
+      </c>
+      <c r="F7" s="12">
+        <f>MAX(0,D7-E7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="13">
+        <f>B7+C7+F7</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>E7+G7</f>
+        <v/>
+      </c>
+      <c r="J7" s="21">
+        <f>IF(H7=0,"-",IF(H7&lt;=5000,"Isento",IF(H7&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="B8" s="12">
+        <f>'Lançamentos Mensais'!L6</f>
+        <v/>
+      </c>
+      <c r="C8" s="12">
+        <f>'Lançamentos Mensais'!I6</f>
+        <v/>
+      </c>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="12">
+        <f>D8*$D$3</f>
+        <v/>
+      </c>
+      <c r="F8" s="12">
+        <f>MAX(0,D8-E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="13">
+        <f>B8+C8+F8</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>E8+G8</f>
+        <v/>
+      </c>
+      <c r="J8" s="21">
+        <f>IF(H8=0,"-",IF(H8&lt;=5000,"Isento",IF(H8&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B9" s="12">
+        <f>'Lançamentos Mensais'!L7</f>
+        <v/>
+      </c>
+      <c r="C9" s="12">
+        <f>'Lançamentos Mensais'!I7</f>
+        <v/>
+      </c>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="12">
+        <f>D9*$D$3</f>
+        <v/>
+      </c>
+      <c r="F9" s="12">
+        <f>MAX(0,D9-E9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="13">
+        <f>B9+C9+F9</f>
+        <v/>
+      </c>
+      <c r="I9" s="13">
+        <f>E9+G9</f>
+        <v/>
+      </c>
+      <c r="J9" s="21">
+        <f>IF(H9=0,"-",IF(H9&lt;=5000,"Isento",IF(H9&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Maio</t>
+        </is>
+      </c>
+      <c r="B10" s="12">
+        <f>'Lançamentos Mensais'!L8</f>
+        <v/>
+      </c>
+      <c r="C10" s="12">
+        <f>'Lançamentos Mensais'!I8</f>
+        <v/>
+      </c>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="12">
+        <f>D10*$D$3</f>
+        <v/>
+      </c>
+      <c r="F10" s="12">
+        <f>MAX(0,D10-E10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="13">
+        <f>B10+C10+F10</f>
+        <v/>
+      </c>
+      <c r="I10" s="13">
+        <f>E10+G10</f>
+        <v/>
+      </c>
+      <c r="J10" s="21">
+        <f>IF(H10=0,"-",IF(H10&lt;=5000,"Isento",IF(H10&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Junho</t>
+        </is>
+      </c>
+      <c r="B11" s="12">
+        <f>'Lançamentos Mensais'!L9</f>
+        <v/>
+      </c>
+      <c r="C11" s="12">
+        <f>'Lançamentos Mensais'!I9</f>
+        <v/>
+      </c>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="12">
+        <f>D11*$D$3</f>
+        <v/>
+      </c>
+      <c r="F11" s="12">
+        <f>MAX(0,D11-E11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="13">
+        <f>B11+C11+F11</f>
+        <v/>
+      </c>
+      <c r="I11" s="13">
+        <f>E11+G11</f>
+        <v/>
+      </c>
+      <c r="J11" s="21">
+        <f>IF(H11=0,"-",IF(H11&lt;=5000,"Isento",IF(H11&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Julho</t>
+        </is>
+      </c>
+      <c r="B12" s="12">
+        <f>'Lançamentos Mensais'!L10</f>
+        <v/>
+      </c>
+      <c r="C12" s="12">
+        <f>'Lançamentos Mensais'!I10</f>
+        <v/>
+      </c>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="12">
+        <f>D12*$D$3</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>MAX(0,D12-E12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="13">
+        <f>B12+C12+F12</f>
+        <v/>
+      </c>
+      <c r="I12" s="13">
+        <f>E12+G12</f>
+        <v/>
+      </c>
+      <c r="J12" s="21">
+        <f>IF(H12=0,"-",IF(H12&lt;=5000,"Isento",IF(H12&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B13" s="12">
+        <f>'Lançamentos Mensais'!L11</f>
+        <v/>
+      </c>
+      <c r="C13" s="12">
+        <f>'Lançamentos Mensais'!I11</f>
+        <v/>
+      </c>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="12">
+        <f>D13*$D$3</f>
+        <v/>
+      </c>
+      <c r="F13" s="12">
+        <f>MAX(0,D13-E13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="13">
+        <f>B13+C13+F13</f>
+        <v/>
+      </c>
+      <c r="I13" s="13">
+        <f>E13+G13</f>
+        <v/>
+      </c>
+      <c r="J13" s="21">
+        <f>IF(H13=0,"-",IF(H13&lt;=5000,"Isento",IF(H13&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>'Lançamentos Mensais'!L12</f>
+        <v/>
+      </c>
+      <c r="C14" s="12">
+        <f>'Lançamentos Mensais'!I12</f>
+        <v/>
+      </c>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="12">
+        <f>D14*$D$3</f>
+        <v/>
+      </c>
+      <c r="F14" s="12">
+        <f>MAX(0,D14-E14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="11" t="n"/>
+      <c r="H14" s="13">
+        <f>B14+C14+F14</f>
+        <v/>
+      </c>
+      <c r="I14" s="13">
+        <f>E14+G14</f>
+        <v/>
+      </c>
+      <c r="J14" s="21">
+        <f>IF(H14=0,"-",IF(H14&lt;=5000,"Isento",IF(H14&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>'Lançamentos Mensais'!L13</f>
+        <v/>
+      </c>
+      <c r="C15" s="12">
+        <f>'Lançamentos Mensais'!I13</f>
+        <v/>
+      </c>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="12">
+        <f>D15*$D$3</f>
+        <v/>
+      </c>
+      <c r="F15" s="12">
+        <f>MAX(0,D15-E15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="13">
+        <f>B15+C15+F15</f>
+        <v/>
+      </c>
+      <c r="I15" s="13">
+        <f>E15+G15</f>
+        <v/>
+      </c>
+      <c r="J15" s="21">
+        <f>IF(H15=0,"-",IF(H15&lt;=5000,"Isento",IF(H15&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Novembro</t>
+        </is>
+      </c>
+      <c r="B16" s="12">
+        <f>'Lançamentos Mensais'!L14</f>
+        <v/>
+      </c>
+      <c r="C16" s="12">
+        <f>'Lançamentos Mensais'!I14</f>
+        <v/>
+      </c>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="12">
+        <f>D16*$D$3</f>
+        <v/>
+      </c>
+      <c r="F16" s="12">
+        <f>MAX(0,D16-E16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="13">
+        <f>B16+C16+F16</f>
+        <v/>
+      </c>
+      <c r="I16" s="13">
+        <f>E16+G16</f>
+        <v/>
+      </c>
+      <c r="J16" s="21">
+        <f>IF(H16=0,"-",IF(H16&lt;=5000,"Isento",IF(H16&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Dezembro</t>
+        </is>
+      </c>
+      <c r="B17" s="12">
+        <f>'Lançamentos Mensais'!L15</f>
+        <v/>
+      </c>
+      <c r="C17" s="12">
+        <f>'Lançamentos Mensais'!I15</f>
+        <v/>
+      </c>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="12">
+        <f>D17*$D$3</f>
+        <v/>
+      </c>
+      <c r="F17" s="12">
+        <f>MAX(0,D17-E17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="13">
+        <f>B17+C17+F17</f>
+        <v/>
+      </c>
+      <c r="I17" s="13">
+        <f>E17+G17</f>
+        <v/>
+      </c>
+      <c r="J17" s="21">
+        <f>IF(H17=0,"-",IF(H17&lt;=5000,"Isento",IF(H17&lt;=7350,"Redução parcial","Tabela cheia")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL ANO</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>SUM(B6:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>SUM(C6:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>SUM(D6:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="15">
+        <f>SUM(E6:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="15">
+        <f>SUM(F6:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="15">
+        <f>SUM(G6:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="15">
+        <f>SUM(H6:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="15">
+        <f>SUM(I6:I17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Como preencher: 'MEI faturamento' = o que sua empresa faturou no mês. A planilha estima a parte isenta</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>(pela presunção) e a parte tributável. 'Bolsa' é isenta (não entra no tributável). Airbnb e outro aluguel</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>vêm das abas/colunas já preenchidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Atenção: o carnê-leão MENSAL (aba Lançamentos, coluna 'IR a pagar') incide só sobre os ALUGUÉIS (PF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>A parte tributável do MEI é acertada na DECLARAÇÃO ANUAL. Como você tem várias fontes, pode haver</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>imposto a pagar no ajuste anual mesmo com DARFs mensais zerados — confirme o número anual com apoio profissional.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>